<commit_message>
feat(F-NAR-019): ATOM-AUT.RAN.001-05 La voiture rouge
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.RAN.001-05.xlsx
+++ b/stories/arbres/ATOM-AUT.RAN.001-05.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre, lumière de miel, odeur d'orange, merle sur la gouttière</t>
+          <t>chambre, odeur d'orange, merle sur la gouttière, caisse à éclat d'écorce</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut l'histoire au lit avec sa voiture rouge, et voir le merle. Les autres voitures recouvrent la rouge. Il les met dans la caisse pour chercher. La rouge apparaît. Rideau, orange, merle.</t>
+          <t>Le merle glisse sur le rideau. Sur la caisse, un éclat d'écorce luit. Victorino veut la rouge sur l'oreiller, maintenant, pour l'histoire. Il ramasse toute la pile : clac, l'éclat disparaît. Papa s'accroupit. Une par une. Merci vécu. Il refuse de foncer. Sous le lit, l'éclat d'écorce reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une odeur d'orange entre dans la chambre. Maman a pelé un fruit, dans la cuisine. La lumière est couleur de miel. Une abeille bourdonne dehors. Puis elle s'en va. Tu as entendu l'abeille, Victorino ? Oui, papa, elle est partie. Le rideau est à moitié fermé. Un merle est sur la gouttière. On l'entend un peu. Il chante tout doux. Le tapis de la chambre est épais. En ce moment, Victorino est à genoux. Il a des voitures rouges et bleues. Il fait une route. La route va de la fenêtre jusqu'au lit. Vroom. Ta route est longue. La voiture rouge avance en tête. Une voiture bleue la suit. Les roues font un petit bruit. Victorino pose les mains en pont. C'est un garage, papa. Un garage au bord de la route. Après, tu racontes, maman ? Oui, au lit, avec le rideau ouvert. La rouge vient avec moi. Victorino la pousse vers le lit. D'autres voitures se poussent. La bleue passe par-dessus. La rouge disparaît sous la pile. Oh. Elles se sont bousculées. Où est ma voiture rouge ? Sous le lit, peut-être ? Victorino se penche. De la poussière, un chausson. Pas de rouge. Dans le garage ? Il ouvre ses deux mains. Le pont de doigts est vide. Elle est perdue. La route est encore au sol. Je veux voir dessous. Victorino prend une voiture bleue. Il la pose dans la caisse. Toc. Le bois glisse un peu.</t>
+          <t>Une ombre d'oiseau glisse sur le rideau. Le merle est sur la gouttière. Au pied du lit, la caisse en bois attend. Un éclat d'écorce luit sur le couvercle. Il brille, papa. Tu le vois, sur le bois ? L'air sent l'orange, depuis la cuisine. J'ai pelé un fruit, Victorino. Le tapis de la chambre est épais. Des voitures rouges et bleues attendent. La rouge va jusqu'au lit, maintenant ! Avec le rideau ouvert, pour l'histoire ? Oui, elle vient sur l'oreiller. Ta route est longue, jusqu'au lit. En ce moment, Victorino pousse la rouge. Les roues font un petit bruit sec. Une bleue la suit, trop près. D'autres voitures se poussent vers le lit. La bleue passe par-dessus la pile. La rouge disparaît sous les toits. Oh ! Le sourire de Victorino disparaît. Où est ma voiture rouge ? Sous le lit, peut-être ? Il se penche, trop vite. De la poussière, un chausson. Pas de rouge. Je prends toute la pile ! Il ramasse les voitures d'un coup. La pile glisse, clac, contre la caisse. Le couvercle bascule. L'éclat d'écorce disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elles se sont bousculées. Elle est perdue.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une odeur d'orange entre dans la chambre. Maman a pelé un fruit, dans la cuisine. La lumière est couleur de miel. Une abeille bourdonne dehors. Puis elle s'en va. Tu as entendu l'abeille, Victorino ? Oui, papa, elle est partie. Le rideau est à moitié fermé. Un merle est sur la gouttière. On l'entend un peu. Il chante tout doux. Le tapis de la chambre est épais. En ce moment, Victorino est à genoux. Il a des voitures rouges et bleues. Il fait une route. La route va de la fenêtre jusqu'au lit. Vroom. Ta route est longue. La voiture rouge avance en tête. Une voiture bleue la suit. Les roues font un petit bruit. Victorino pose les mains en pont. C'est un garage, papa. Un garage au bord de la route. Après, tu racontes, maman ? Oui, au lit, avec le rideau ouvert. La rouge vient avec moi. Victorino la pousse vers le lit. D'autres voitures se poussent. La bleue passe par-dessus. La rouge disparaît sous la pile. Oh. Elles se sont bousculées. Où est ma voiture rouge ? Sous le lit, peut-être ? Victorino se penche. De la poussière, un chausson. Pas de rouge. Dans le garage ? Il ouvre ses deux mains. Le pont de doigts est vide. Elle est perdue. La route est encore au sol. Je veux voir dessous. Victorino prend une voiture bleue. Il la pose dans la caisse. Toc. Le bois glisse un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une ombre d'oiseau glisse sur le rideau. Le merle est sur la gouttière. Au pied du lit, la caisse en bois attend. Un &lt;emphasis level="moderate"&gt;éclat d'écorce&lt;/emphasis&gt; luit sur le couvercle. Il brille, papa. Tu le vois, sur le bois ? L'air sent l'orange, depuis la cuisine. J'ai pelé un fruit, Victorino. Le tapis de la chambre est épais. Des voitures rouges et bleues attendent. La rouge va jusqu'au lit, maintenant ! Avec le rideau ouvert, pour l'histoire ? Oui, elle vient sur l'oreiller. Ta route est longue, jusqu'au lit. En ce moment, Victorino pousse la rouge. Les roues font un petit bruit sec. Une bleue la suit, trop près. D'autres voitures se poussent vers le lit. La bleue passe par-dessus la pile. La rouge disparaît sous les toits. Oh ! Le sourire de Victorino disparaît. Où est ma voiture rouge ? Sous le lit, peut-être ? Il se penche, trop vite. De la poussière, un chausson. Pas de rouge. Je prends toute la pile ! Il ramasse les voitures d'un coup. La pile glisse, clac, contre la caisse. Le couvercle bascule. L'éclat d'écorce disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elles se sont bousculées. Elle est perdue.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>César joue dans sa chambre. Papa est près de la fenêtre. César a des voitures. Les voitures sont rouges et bleues. César fait une route. Les voitures font vroom. Puis le jeu est fini. Papa dit : c'est l'heure de &lt;emphasis&gt;ranger&lt;/emphasis&gt;. César prend une voiture. Il la met dans la caisse. Il prend une autre voiture. Il la met dans la caisse. Encore une voiture. Dans la caisse. La caisse est pleine. Le tapis est vide. Ranger, c'est mettre dans la caisse. Papa dit : merci César. César ferme la caisse. Ça fait toc. Le sol est libre. Papa sourit. [pause]</t>
+          <t>Une ombre d'oiseau glisse sur le rideau. Le merle est sur la gouttière. Au pied du lit, la caisse en bois attend. Un &lt;emphasis&gt;éclat d'écorce&lt;/emphasis&gt; luit sur le couvercle. Il brille, papa. Tu le vois, sur le bois ? L'air sent l'orange, depuis la cuisine. J'ai pelé un fruit, Victorino. Le tapis de la chambre est épais. Des voitures rouges et bleues attendent. La rouge va jusqu'au lit, maintenant ! Avec le rideau ouvert, pour l'histoire ? Oui, elle vient sur l'oreiller. Ta route est longue, jusqu'au lit. En ce moment, Victorino pousse la rouge. Les roues font un petit bruit sec. Une bleue la suit, trop près. D'autres voitures se poussent vers le lit. La bleue passe par-dessus la pile. La rouge disparaît sous les toits. Oh ! Le sourire de Victorino disparaît. Où est ma voiture rouge ? Sous le lit, peut-être ? Il se penche, trop vite. De la poussière, un chausson. Pas de rouge. Je prends toute la pile ! Il ramasse les voitures d'un coup. La pile glisse, clac, contre la caisse. Le couvercle bascule. L'éclat d'écorce disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Elles se sont bousculées. Elle est perdue. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>ranger</t>
+          <t>éclat d'écorce</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,57 +1321,53 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_rouge_sur_l_oreiller_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une odeur d'orange entre dans la chambre.
-narrateur|Maman a pelé un fruit, dans la cuisine.
-narrateur|La lumière est couleur de miel.
-narrateur|Une abeille bourdonne dehors.
-narrateur|Puis elle s'en va.
-papa|Tu as entendu l'abeille, Victorino ?
-enfant-m|Oui, papa, elle est partie.
-narrateur|Le rideau est à moitié fermé.
-narrateur|Un merle est sur la gouttière.
-narrateur|On l'entend un peu.
-maman|Il chante tout doux.
+          <t>narrateur|Une ombre d'oiseau glisse sur le rideau.
+narrateur|Le merle est sur la gouttière.
+narrateur|Au pied du lit, la caisse en bois attend.
+narrateur|Un éclat d'écorce luit sur le couvercle.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le bois ?
+narrateur|L'air sent l'orange, depuis la cuisine.
+maman|J'ai pelé un fruit, Victorino.
 narrateur|Le tapis de la chambre est épais.
-narrateur|En ce moment, Victorino est à genoux.
-narrateur|Il a des voitures rouges et bleues.
-narrateur|Il fait une route.
-narrateur|La route va de la fenêtre jusqu'au lit.
-enfant-m|Vroom.
-papa|Ta route est longue.
-narrateur|La voiture rouge avance en tête.
-narrateur|Une voiture bleue la suit.
-narrateur|Les roues font un petit bruit.
-narrateur|Victorino pose les mains en pont.
-enfant-m|C'est un garage, papa.
-papa|Un garage au bord de la route.
-enfant-m|Après, tu racontes, maman ?
-maman|Oui, au lit, avec le rideau ouvert.
-enfant-m|La rouge vient avec moi.
-narrateur|Victorino la pousse vers le lit.
-narrateur|D'autres voitures se poussent.
-narrateur|La bleue passe par-dessus.
-narrateur|La rouge disparaît sous la pile.
-enfant-m|Oh.
-papa|Elles se sont bousculées.
+narrateur|Des voitures rouges et bleues attendent.
+enfant-m|La rouge va jusqu'au lit, maintenant !
+maman|Avec le rideau ouvert, pour l'histoire ?
+enfant-m|Oui, elle vient sur l'oreiller.
+papa|Ta route est longue, jusqu'au lit.
+narrateur|En ce moment, Victorino pousse la rouge.
+narrateur|Les roues font un petit bruit sec.
+narrateur|Une bleue la suit, trop près.
+narrateur|D'autres voitures se poussent vers le lit.
+narrateur|La bleue passe par-dessus la pile.
+narrateur|La rouge disparaît sous les toits.
+enfant-m|Oh !
+narrateur|Le sourire de Victorino disparaît.
 enfant-m|Où est ma voiture rouge ?
 maman|Sous le lit, peut-être ?
-narrateur|Victorino se penche.
+narrateur|Il se penche, trop vite.
 narrateur|De la poussière, un chausson.
 narrateur|Pas de rouge.
-enfant-m|Dans le garage ?
-narrateur|Il ouvre ses deux mains.
-narrateur|Le pont de doigts est vide.
-enfant-m|Elle est perdue.
-papa|La route est encore au sol.
-enfant-m|Je veux voir dessous.
-narrateur|Victorino prend une voiture bleue.
-narrateur|Il la pose dans la caisse.
-narrateur|Toc.
-narrateur|Le bois glisse un peu.</t>
+enfant-m|Je prends toute la pile !
+narrateur|Il ramasse les voitures d'un coup.
+narrateur|La pile glisse, clac, contre la caisse.
+narrateur|Le couvercle bascule.
+narrateur|L'éclat d'écorce disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Elles se sont bousculées.
+enfant-m|Elle est perdue.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>rideau,merle,orange,voitures</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1399,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino cherche sa voiture rouge. Où est-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino cherche sa &lt;emphasis level="moderate"&gt;voiture rouge&lt;/emphasis&gt;. Où est-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Après le jeu, que fait César ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino cherche sa &lt;emphasis&gt;voiture rouge&lt;/emphasis&gt;. Où est-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1471,7 +1467,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,7 +1478,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1493,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>voiture rouge</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1539,17 +1539,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_est_sous_les_autres; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1582,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Une autre bleue va dans la caisse. Toc. Tu regardes bien sous la route ? Oui, maman. Un bout de tapis reparaît. Encore une, tout doux. Victorino soulève une voiture noire. Un toit rouge brille dessous. Ma rouge ! La voiture rouge était sous les autres. Elle sent encore le tapis. Victorino la tient dans la paume. Le métal est un peu froid. Merci, tu l'as trouvée. Te voilà, petite rouge. Elle était dessous. Les dernières voitures vont dans la caisse. Le chemin du lit est libre. Le merle chante encore un peu.</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes bien sous la route ? Oui, papa. Victorino pose une bleue dans la caisse. Toc. Un bout de tapis reparaît. Une par une, Victorino. Il soulève une voiture noire. Un toit rouge brille dessous. Ma rouge ! La voiture rouge était sous les autres. Elle sent le tapis, un peu froide. Merci, tu l'as trouvée. Le couvercle de la caisse se rassoit. L'éclat d'écorce reparaît, pâle. Il est revenu. Te voilà, petite rouge. Elle était dessous. Victorino la tient dans la paume. Il essuie le tapis du toit, du pouce. Le chemin du lit est presque libre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Une autre bleue va dans la caisse. Toc. Tu regardes bien sous la route ? Oui, maman. Un bout de tapis reparaît. Encore une, tout doux. Victorino soulève une voiture noire. Un toit rouge brille dessous. Ma rouge ! La voiture rouge était sous les autres. Elle sent encore le tapis. Victorino la tient dans la paume. Le métal est un peu froid. Merci, tu l'as trouvée. Te voilà, petite rouge. Elle était dessous. Les dernières voitures vont dans la caisse. Le chemin du lit est libre. Le merle chante encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Tu regardes bien sous la route ? Oui, papa. Victorino pose une bleue dans la caisse. Toc. Un bout de tapis reparaît. Une par une, Victorino. Il soulève une voiture noire. Un toit rouge brille dessous. Ma rouge ! La voiture rouge était sous les autres. Elle sent le tapis, un peu froide. Merci, tu l'as trouvée. Le couvercle de la caisse se rassoit. L'&lt;emphasis level="moderate"&gt;éclat d'écorce&lt;/emphasis&gt; reparaît, pâle. Il est revenu. Te voilà, petite rouge. Elle était dessous. Victorino la tient dans la paume. Il essuie le tapis du toit, du pouce. Le chemin du lit est presque libre.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>César a rangé. Les voitures sont dans la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Le tapis est libre. Papa est là. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes bien sous la route ? Oui, papa. Victorino pose une bleue dans la caisse. Toc. Un bout de tapis reparaît. Une par une, Victorino. Il soulève une voiture noire. Un toit rouge brille dessous. Ma rouge ! La voiture rouge était sous les autres. Elle sent le tapis, un peu froide. Merci, tu l'as trouvée. Le couvercle de la caisse se rassoit. L'&lt;emphasis&gt;éclat d'écorce&lt;/emphasis&gt; reparaît, pâle. Il est revenu. Te voilà, petite rouge. Elle était dessous. Victorino la tient dans la paume. Il essuie le tapis du toit, du pouce. Le chemin du lit est presque libre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1650,7 +1650,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>éclat d'écorce</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1687,16 +1687,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1721,30 +1721,37 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=une_par_une_le_toit_rouge_reparaît; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Une autre bleue va dans la caisse.
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu regardes bien sous la route ?
+enfant-m|Oui, papa.
+narrateur|Victorino pose une bleue dans la caisse.
 narrateur|Toc.
-maman|Tu regardes bien sous la route ?
-enfant-m|Oui, maman.
 narrateur|Un bout de tapis reparaît.
-papa|Encore une, tout doux.
-narrateur|Victorino soulève une voiture noire.
+maman|Une par une, Victorino.
+narrateur|Il soulève une voiture noire.
 narrateur|Un toit rouge brille dessous.
 enfant-m|Ma rouge !
 narrateur|La voiture rouge était sous les autres.
-narrateur|Elle sent encore le tapis.
-narrateur|Victorino la tient dans la paume.
-narrateur|Le métal est un peu froid.
+narrateur|Elle sent le tapis, un peu froide.
 papa|Merci, tu l'as trouvée.
+narrateur|Le couvercle de la caisse se rassoit.
+narrateur|L'éclat d'écorce reparaît, pâle.
+enfant-m|Il est revenu.
 maman|Te voilà, petite rouge.
 enfant-m|Elle était dessous.
-narrateur|Les dernières voitures vont dans la caisse.
-narrateur|Le chemin du lit est libre.
-narrateur|Le merle chante encore un peu.</t>
+narrateur|Victorino la tient dans la paume.
+narrateur|Il essuie le tapis du toit, du pouce.
+papa|Le chemin du lit est presque libre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>caisse,voitures</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1778,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorino pousse la caisse sous le lit. Le bois glisse tout doucement. On ouvre le rideau ? Oui, tout grand. Le merle est encore sur la gouttière. Il penche la tête. Victorino grimpe sur le lit. La voiture rouge est sur l'oreiller. Je raconte ? Oui, maman. Maman s'assoit au bord. Sa voix est basse, tout près. Tu veux un quartier d'orange ? Oui, papa. L'orange sent fort, sucrée. Le jus brille un peu sur le doigt. Le merle écoute aussi, on dirait.</t>
+          <t>Les dernières voitures restent en tas. Je les pousse toutes, maintenant ! Il avance les mains vers le tas. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Victorino observe la caisse, écoute la chambre. Sur le couvercle, l'éclat d'écorce luit. Là, près de l'éclat. Il soulève la dernière bleue, tout près. Rien dessous, seulement le tapis. Les dernières voitures vont dans la caisse. Toc. On ouvre le rideau ? Oui, tout grand. La rouge vient avec toi ? Oui, sur l'oreiller. Victorino pousse la caisse sous le lit. Le bois glisse, l'éclat d'écorce aussi. Un filet de soleil entre sur le tapis. Victorino grimpe sur le lit. La voiture rouge est sur l'oreiller. Je raconte ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorino pousse la caisse sous le lit. Le bois glisse tout doucement. On ouvre le rideau ? Oui, tout grand. Le merle est encore sur la gouttière. Il penche la tête. Victorino grimpe sur le lit. La voiture rouge est sur l'oreiller. Je raconte ? Oui, maman. Maman s'assoit au bord. Sa voix est basse, tout près. Tu veux un quartier d'orange ? Oui, papa. L'orange sent fort, sucrée. Le jus brille un peu sur le doigt. Le merle écoute aussi, on dirait.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les dernières voitures restent en tas. Je les pousse toutes, maintenant ! Il avance les mains vers le tas. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Victorino observe la caisse, écoute la chambre. Sur le couvercle, l'&lt;emphasis level="moderate"&gt;éclat d'écorce&lt;/emphasis&gt; luit. Là, près de l'éclat. Il soulève la dernière bleue, tout près. Rien dessous, seulement le tapis. Les dernières voitures vont dans la caisse. Toc. On ouvre le rideau ? Oui, tout grand. La rouge vient avec toi ? Oui, sur l'oreiller. Victorino pousse la caisse sous le lit. Le bois glisse, l'éclat d'écorce aussi. Un filet de soleil entre sur le tapis. Victorino grimpe sur le lit. La voiture rouge est sur l'oreiller. Je raconte ? Oui, maman.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>César ferme la &lt;emphasis&gt;caisse&lt;/emphasis&gt;. Papa lui tend l'eau. [pause]</t>
+          <t>Les dernières voitures restent en tas. Je les pousse toutes, maintenant ! Il avance les mains vers le tas. Puis il s'arrête net. Il refuse de foncer. Attends, je regarde. Papa attend, sans parler. Victorino observe la caisse, écoute la chambre. Sur le couvercle, l'&lt;emphasis&gt;éclat d'écorce&lt;/emphasis&gt; luit. Là, près de l'éclat. Il soulève la dernière bleue, tout près. Rien dessous, seulement le tapis. Les dernières voitures vont dans la caisse. Toc. On ouvre le rideau ? Oui, tout grand. La rouge vient avec toi ? Oui, sur l'oreiller. Victorino pousse la caisse sous le lit. Le bois glisse, l'éclat d'écorce aussi. Un filet de soleil entre sur le tapis. Victorino grimpe sur le lit. La voiture rouge est sur l'oreiller. Je raconte ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1828,7 +1835,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1836,10 +1843,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1862,30 +1869,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>caisse</t>
+          <t>éclat d'écorce</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1894,10 +1901,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,26 +1915,43 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorino pousse la caisse sous le lit.
-narrateur|Le bois glisse tout doucement.
-enfant-m|On ouvre le rideau ?
-papa|Oui, tout grand.
-narrateur|Le merle est encore sur la gouttière.
-narrateur|Il penche la tête.
+          <t>narrateur|Les dernières voitures restent en tas.
+enfant-m|Je les pousse toutes, maintenant !
+narrateur|Il avance les mains vers le tas.
+narrateur|Puis il s'arrête net.
+narrateur|Il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Victorino observe la caisse, écoute la chambre.
+narrateur|Sur le couvercle, l'éclat d'écorce luit.
+enfant-m|Là, près de l'éclat.
+narrateur|Il soulève la dernière bleue, tout près.
+narrateur|Rien dessous, seulement le tapis.
+narrateur|Les dernières voitures vont dans la caisse.
+narrateur|Toc.
+maman|On ouvre le rideau ?
+enfant-m|Oui, tout grand.
+papa|La rouge vient avec toi ?
+enfant-m|Oui, sur l'oreiller.
+narrateur|Victorino pousse la caisse sous le lit.
+narrateur|Le bois glisse, l'éclat d'écorce aussi.
+narrateur|Un filet de soleil entre sur le tapis.
 narrateur|Victorino grimpe sur le lit.
 narrateur|La voiture rouge est sur l'oreiller.
 maman|Je raconte ?
-enfant-m|Oui, maman.
-narrateur|Maman s'assoit au bord.
-narrateur|Sa voix est basse, tout près.
-papa|Tu veux un quartier d'orange ?
-enfant-m|Oui, papa.
-narrateur|L'orange sent fort, sucrée.
-narrateur|Le jus brille un peu sur le doigt.
-narrateur|Le merle écoute aussi, on dirait.</t>
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>caisse,rideau</t>
         </is>
       </c>
     </row>
@@ -1954,17 +1978,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La rouge est sur l'oreiller. Toi aussi, tu es bien. Bravo, tu l'as retrouvée. L'odeur d'orange reste dans la chambre. Le merle se tait, tout doux.</t>
+          <t>Maman s'assoit au bord du lit. Sa voix est basse, tout près. Tu veux un quartier d'orange ? Oui, papa. L'orange sent fort, sucrée. Le jus brille un peu sur le doigt. La rouge a un petit éclat. Un éclat d'écorce tient sur le toit. Tu le vois, comme sur la caisse ? Oui, maman. Le merle penche la tête, dehors. Sous le lit, l'éclat d'écorce reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La rouge est sur l'oreiller. Toi aussi, tu es bien. Bravo, tu l'as retrouvée. L'odeur d'orange reste dans la chambre. Le merle se tait, tout doux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Maman s'assoit au bord du lit. Sa voix est basse, tout près. Tu veux un quartier d'orange ? Oui, papa. L'orange sent fort, sucrée. Le jus brille un peu sur le doigt. La rouge a un petit éclat. Un &lt;emphasis level="moderate"&gt;éclat d'écorce&lt;/emphasis&gt; tient sur le toit. Tu le vois, comme sur la caisse ? Oui, maman. Le merle penche la tête, dehors. Sous le lit, l'éclat d'écorce reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Maman s'assoit au bord du lit. Sa voix est basse, tout près. Tu veux un quartier d'orange ? Oui, papa. L'orange sent fort, sucrée. Le jus brille un peu sur le doigt. La rouge a un petit éclat. Un &lt;emphasis&gt;éclat d'écorce&lt;/emphasis&gt; tient sur le toit. Tu le vois, comme sur la caisse ? Oui, maman. Le merle penche la tête, dehors. Sous le lit, l'éclat d'écorce reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2035,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2055,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2069,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'écorce</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2092,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,28 +2105,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_toit_rouge; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|La rouge est sur l'oreiller.
-maman|Toi aussi, tu es bien.
-papa|Bravo, tu l'as retrouvée.
-narrateur|L'odeur d'orange reste dans la chambre.
-narrateur|Le merle se tait, tout doux.</t>
+          <t>narrateur|Maman s'assoit au bord du lit.
+narrateur|Sa voix est basse, tout près.
+papa|Tu veux un quartier d'orange ?
+enfant-m|Oui, papa.
+narrateur|L'orange sent fort, sucrée.
+narrateur|Le jus brille un peu sur le doigt.
+enfant-m|La rouge a un petit éclat.
+narrateur|Un éclat d'écorce tient sur le toit.
+maman|Tu le vois, comme sur la caisse ?
+enfant-m|Oui, maman.
+narrateur|Le merle penche la tête, dehors.
+narrateur|Sous le lit, l'éclat d'écorce reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>orange,merle</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2211,6 +2255,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>